<commit_message>
scan: seg1 2026-09-29 01:42 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq2_2026-09-24.xlsx
+++ b/output/full_scan/batch_seq2_2026-09-24.xlsx
@@ -1174,7 +1174,7 @@
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>947.2159540596946</v>
+        <v>907.2159540596946</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>77.40000000000001</v>
@@ -3177,21 +3177,21 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>1815</v>
+        <v>2301</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>富喬</t>
+          <t>光寶科</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>608.5170309436568</v>
+        <v>604.346243903242</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>116</v>
+        <v>287</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,16 +3202,16 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>50.20592836180932</v>
+        <v>53.66341765473977</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>31.51267897007891</v>
+        <v>29.5405773760245</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.4091265424535423</v>
+        <v>0.4255381368334286</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-1.896972719138102</v>
+        <v>-2.40364639860854</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>2301</v>
+        <v>2441</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>光寶科</t>
+          <t>超豐</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>604.346243903242</v>
+        <v>601.6502080181851</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>287</v>
+        <v>124</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,13 +3255,13 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>53.66341765473977</v>
+        <v>56.93159659709492</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>29.5405773760245</v>
+        <v>16.38853723654727</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.4255381368334286</v>
+        <v>0.6563858128763391</v>
       </c>
       <c r="K53" s="2" t="n">
         <v>1</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-2.40364639860854</v>
+        <v>1.354916534943151</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>2441</v>
+        <v>2107</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>超豐</t>
+          <t>厚生</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>601.6502080181851</v>
+        <v>599.0139968055466</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>124</v>
+        <v>26.95</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,16 +3308,16 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>56.93159659709492</v>
+        <v>56.19444630633507</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>16.38853723654727</v>
+        <v>23.42866125198688</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.6563858128763391</v>
+        <v>0.8317861121425919</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>1.354916534943151</v>
+        <v>-0.0218276706329851</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>2107</v>
+        <v>2421</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>厚生</t>
+          <t>建準</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>599.0139968055466</v>
+        <v>592.6842801328203</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>26.95</v>
+        <v>167</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,16 +3361,16 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>56.19444630633507</v>
+        <v>56.36437442007536</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>23.42866125198688</v>
+        <v>16.98581197336325</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.8317861121425919</v>
+        <v>0.3693269264607346</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-0.0218276706329851</v>
+        <v>-0.8673451579435074</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>2421</v>
+        <v>2104</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>建準</t>
+          <t>國際中橡</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>592.6842801328203</v>
+        <v>589.6716709476325</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>167</v>
+        <v>11.15</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,16 +3414,16 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>56.36437442007536</v>
+        <v>59.45129495411348</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>16.98581197336325</v>
+        <v>29.55860870134153</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.3693269264607346</v>
+        <v>2.201451231272236</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-0.8673451579435074</v>
+        <v>0.0880937764864289</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>volume_break, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>2104</v>
+        <v>1904</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>國際中橡</t>
+          <t>正隆</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>589.6716709476325</v>
+        <v>585.9969410619888</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>11.15</v>
+        <v>24.9</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,16 +3467,16 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>59.45129495411348</v>
+        <v>53.87496287507386</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>29.55860870134153</v>
+        <v>28.12096990264753</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>2.201451231272236</v>
+        <v>0.6942681600017268</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.0880937764864289</v>
+        <v>-0.0679101660109234</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>1904</v>
+        <v>2338</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>正隆</t>
+          <t>光罩</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>585.9969410619888</v>
+        <v>581.8562867615966</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>24.9</v>
+        <v>47.1</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,16 +3520,16 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>53.87496287507386</v>
+        <v>58.03948122317059</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>28.12096990264753</v>
+        <v>39.2313854154655</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.6942681600017268</v>
+        <v>0.2517450244329172</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.0679101660109234</v>
+        <v>0.2991476719303518</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>2338</v>
+        <v>2399</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>光罩</t>
+          <t>映泰</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>581.8562867615966</v>
+        <v>580.1434711704227</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>47.1</v>
+        <v>47.3</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,13 +3573,13 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>58.03948122317059</v>
+        <v>53.8991072324332</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>39.2313854154655</v>
+        <v>19.18509183547802</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.2517450244329172</v>
+        <v>0.3239170823003393</v>
       </c>
       <c r="K59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.2991476719303518</v>
+        <v>-0.0179219471292723</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>2399</v>
+        <v>2424</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>映泰</t>
+          <t>隴華</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>580.1434711704227</v>
+        <v>576.4181644897611</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>47.3</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,13 +3626,13 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>53.8991072324332</v>
+        <v>49.63413613368842</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>19.18509183547802</v>
+        <v>21.40773066113696</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.3239170823003393</v>
+        <v>0.58268884415722</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.0179219471292723</v>
+        <v>0.0501257320161909</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>2424</v>
+        <v>2038</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>隴華</t>
+          <t>海光</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>576.4181644897611</v>
+        <v>571.6575452231314</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>8.199999999999999</v>
+        <v>12.55</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>49.63413613368842</v>
+        <v>54.64959770622918</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>21.40773066113696</v>
+        <v>27.54805260943758</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.58268884415722</v>
+        <v>3.476784031269073</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>0</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.0501257320161909</v>
+        <v>0.0257841614736626</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>macd_golden_cross, volume_break, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>2038</v>
+        <v>2351</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>海光</t>
+          <t>順德</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>571.6575452231314</v>
+        <v>571.4532672135879</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>12.55</v>
+        <v>219.5</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,16 +3732,16 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>54.64959770622918</v>
+        <v>47.81893156998148</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>27.54805260943758</v>
+        <v>29.57893331786734</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>3.476784031269073</v>
+        <v>0.822446880628226</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.0257841614736626</v>
+        <v>-3.910376432301448</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, volume_break, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>2351</v>
+        <v>1815</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>順德</t>
+          <t>富喬</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>571.4532672135879</v>
+        <v>568.5170309436568</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>219.5</v>
+        <v>116</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,16 +3785,16 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>47.81893156998148</v>
+        <v>50.20592836180932</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>29.57893331786734</v>
+        <v>31.51267897007891</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.822446880628226</v>
+        <v>0.4091265424535423</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L63" s="2" t="n">
         <v>0</v>
@@ -3803,11 +3803,11 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-3.910376432301448</v>
+        <v>-1.896972719138102</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -5085,21 +5085,21 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>1785</v>
+        <v>2208</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>光洋科</t>
+          <t>台船</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>458.0836760282951</v>
+        <v>453.8985888713039</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>95.8</v>
+        <v>19.4</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>39.33347979389713</v>
+        <v>55.3257968146044</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>26.8883656200478</v>
+        <v>22.05186260069619</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.7104465843872415</v>
+        <v>0.7558225980049488</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.3327942130494321</v>
+        <v>0.0742220764531602</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>2208</v>
+        <v>2393</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>台船</t>
+          <t>億光</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>453.8985888713039</v>
+        <v>447.4667127234046</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>19.4</v>
+        <v>63.4</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,16 +5163,16 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>55.3257968146044</v>
+        <v>48.46569377816383</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>22.05186260069619</v>
+        <v>11.08529073392815</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.7558225980049488</v>
+        <v>1.300608595932826</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L89" s="2" t="n">
         <v>0</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.0742220764531602</v>
+        <v>0.0349018032715383</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>2393</v>
+        <v>1710</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>億光</t>
+          <t>東聯</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>447.4667127234046</v>
+        <v>447.1977816965119</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>63.4</v>
+        <v>16.4</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,16 +5216,16 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>48.46569377816383</v>
+        <v>54.66097982099056</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>11.08529073392815</v>
+        <v>26.87481327581776</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>1.300608595932826</v>
+        <v>0.6202075356997018</v>
       </c>
       <c r="K90" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.0349018032715383</v>
+        <v>0.0283285405145085</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>1710</v>
+        <v>1614</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>東聯</t>
+          <t>三洋電</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>447.1977816965119</v>
+        <v>446.0100917828321</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>16.4</v>
+        <v>31.15</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,13 +5269,13 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>54.66097982099056</v>
+        <v>56.37527112948978</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>26.87481327581776</v>
+        <v>26.7161312942137</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.6202075356997018</v>
+        <v>0.5236319123987626</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>0.0283285405145085</v>
+        <v>0.0477903844214449</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>1614</v>
+        <v>2106</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>三洋電</t>
+          <t>建大</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>446.0100917828321</v>
+        <v>437.3727309333153</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>31.15</v>
+        <v>16.65</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,16 +5322,16 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>56.37527112948978</v>
+        <v>42.50155324750998</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>26.7161312942137</v>
+        <v>22.2041153467602</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.5236319123987626</v>
+        <v>0.1993209185384439</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L92" s="2" t="n">
         <v>0</v>
@@ -5340,51 +5340,51 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.0477903844214449</v>
+        <v>0.0101202395393836</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>2106</v>
+        <v>1589</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>建大</t>
+          <t>永冠-KY</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>437.3727309333153</v>
+        <v>436.2437654589683</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>16.65</v>
+        <v>5.54</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="G93" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>42.50155324750998</v>
+        <v>24.03488264070512</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>22.2041153467602</v>
+        <v>38.86916791888412</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.1993209185384439</v>
+        <v>4.024376545896833</v>
       </c>
       <c r="K93" s="2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="L93" s="2" t="n">
         <v>0</v>
@@ -5393,51 +5393,51 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>0.0101202395393836</v>
+        <v>0.0987299345354202</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, obv_uptrend</t>
+          <t>volume_break, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>1589</v>
+        <v>2009</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>永冠-KY</t>
+          <t>第一銅</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>436.2437654589683</v>
+        <v>435.0610665187907</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>5.54</v>
+        <v>39.15</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G94" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>24.03488264070512</v>
+        <v>47.62274020682705</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>38.86916791888412</v>
+        <v>22.63269151703244</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>4.024376545896833</v>
+        <v>0.4548821519677418</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.0987299345354202</v>
+        <v>-0.0622745405603558</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>2009</v>
+        <v>1731</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>第一銅</t>
+          <t>美吾華</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>435.0610665187907</v>
+        <v>432.6730178963597</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>39.15</v>
+        <v>20.9</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,16 +5481,16 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>47.62274020682705</v>
+        <v>49.94539012669958</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>22.63269151703244</v>
+        <v>12.45688393393229</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.4548821519677418</v>
+        <v>0.7407744247118293</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.0622745405603558</v>
+        <v>0.003893336922151</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>1731</v>
+        <v>1717</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>美吾華</t>
+          <t>長興</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>432.6730178963597</v>
+        <v>426.9108097023167</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>20.9</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,16 +5534,16 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>49.94539012669958</v>
+        <v>48.37106891299786</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>12.45688393393229</v>
+        <v>9.719419490399524</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.7407744247118293</v>
+        <v>0.2905782265316657</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.003893336922151</v>
+        <v>-0.341949402108933</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>1717</v>
+        <v>2408</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>長興</t>
+          <t>南亞科</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>426.9108097023167</v>
+        <v>425.0667721724499</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>71.40000000000001</v>
+        <v>503</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,13 +5587,13 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>48.37106891299786</v>
+        <v>50.98652261854292</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>9.719419490399524</v>
+        <v>13.35158288202788</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.2905782265316657</v>
+        <v>0.6214390799489438</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.341949402108933</v>
+        <v>-1.7994939967812</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>2408</v>
+        <v>2369</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>南亞科</t>
+          <t>菱生</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>425.0667721724499</v>
+        <v>424.3920778015262</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>503</v>
+        <v>31.25</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,16 +5640,16 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>50.98652261854292</v>
+        <v>50.39573472492294</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>13.35158288202788</v>
+        <v>16.88014087372637</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.6214390799489438</v>
+        <v>0.5273223571435459</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-1.7994939967812</v>
+        <v>0.2967965957789135</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>2369</v>
+        <v>2352</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>菱生</t>
+          <t>佳世達</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>424.3920778015262</v>
+        <v>424.2262204859846</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>31.25</v>
+        <v>29</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,16 +5693,16 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>50.39573472492294</v>
+        <v>50.65241521578172</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>16.88014087372637</v>
+        <v>18.77315284939832</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.5273223571435459</v>
+        <v>0.4997094857052206</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L99" s="2" t="n">
         <v>0</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.2967965957789135</v>
+        <v>0.0625257244008772</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5721,21 +5721,21 @@
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>2352</v>
+        <v>2405</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>佳世達</t>
+          <t>輔信</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>424.2262204859846</v>
+        <v>424.088159320306</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>29</v>
+        <v>15.05</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,16 +5746,16 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>50.65241521578172</v>
+        <v>45.53810146645605</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>18.77315284939832</v>
+        <v>20.87364037095257</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.4997094857052206</v>
+        <v>0.7443935630658249</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.0625257244008772</v>
+        <v>0.0689249247390242</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>2405</v>
+        <v>1785</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>輔信</t>
+          <t>光洋科</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>424.088159320306</v>
+        <v>418.0836760282951</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>15.05</v>
+        <v>95.8</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,16 +5799,16 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>45.53810146645605</v>
+        <v>39.33347979389713</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>20.87364037095257</v>
+        <v>26.8883656200478</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.7443935630658249</v>
+        <v>0.7104465843872415</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L101" s="2" t="n">
         <v>0</v>
@@ -5817,11 +5817,11 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.0689249247390242</v>
+        <v>0.3327942130494321</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>

</xml_diff>